<commit_message>
Update daily activity tracker data
</commit_message>
<xml_diff>
--- a/Daily_Activity_Tracker/12600762.xlsx
+++ b/Daily_Activity_Tracker/12600762.xlsx
@@ -23,8 +23,6 @@
     <style:font-face style:name="ArialMT" svg:font-family="ArialMT"/>
     <style:font-face style:name="Calibri" svg:font-family="Calibri"/>
     <style:font-face style:name="Liberation Sans" svg:font-family="'Liberation Sans'" style:font-family-generic="swiss" style:font-pitch="variable"/>
-    <style:font-face style:name="Liberation Serif" svg:font-family="'Liberation Serif'" style:font-family-generic="roman" style:font-pitch="variable"/>
-    <style:font-face style:name="Tahoma" svg:font-family="Tahoma" style:font-family-generic="system" style:font-pitch="variable"/>
   </office:font-face-decls>
   <office:automatic-styles>
     <style:style style:name="co1" style:family="table-column">
@@ -116,7 +114,7 @@
       <style:table-cell-properties fo:padding-bottom="0.071cm" fo:padding-left="0.071cm" fo:padding-right="0.071cm" fo:padding-top="0.035cm" style:vertical-align="bottom"/>
       <style:text-properties fo:color="#000000" style:font-name="Calibri" fo:font-size="11pt" style:font-name-asian="Calibri" style:font-size-asian="11pt" style:font-name-complex="Calibri" style:font-size-complex="11pt"/>
     </style:style>
-    <style:style style:name="Sheet0_cell1" style:family="table-cell" style:parent-style-name="Default">
+    <style:style style:name="ce3" style:family="table-cell" style:parent-style-name="Default">
       <style:table-cell-properties fo:background-color="#ffffff" fo:padding-bottom="0.071cm" fo:padding-left="0.071cm" fo:padding-right="0.071cm" fo:padding-top="0.035cm" style:vertical-align="bottom"/>
       <style:text-properties fo:color="#000000" style:font-name="Calibri" fo:font-size="11pt" style:font-name-asian="Calibri" style:font-size-asian="11pt" style:font-name-complex="Calibri" style:font-size-complex="11pt"/>
     </style:style>
@@ -245,6 +243,10 @@
       <style:text-properties fo:color="#000000" style:font-name="ArialMT" fo:font-size="11pt" style:font-name-asian="ArialMT" style:font-size-asian="11pt" style:font-name-complex="ArialMT" style:font-size-complex="11pt"/>
     </style:style>
     <style:style style:name="Sheet2_cell22" style:family="table-cell" style:parent-style-name="Default">
+      <style:table-cell-properties fo:background-color="#ffffff" fo:border="0.99pt solid #b7b7b7" fo:padding-bottom="0.071cm" fo:padding-left="0.071cm" fo:padding-right="0.071cm" fo:padding-top="0.035cm" style:vertical-align="middle"/>
+      <style:text-properties fo:color="#000000" style:font-name="ArialMT" fo:font-size="11pt" style:font-name-asian="ArialMT" style:font-size-asian="11pt" style:font-name-complex="ArialMT" style:font-size-complex="11pt"/>
+    </style:style>
+    <style:style style:name="ce37" style:family="table-cell" style:parent-style-name="Default" style:data-style-name="N0">
       <style:table-cell-properties fo:background-color="#ffffff" fo:border="0.99pt solid #b7b7b7" fo:padding-bottom="0.071cm" fo:padding-left="0.071cm" fo:padding-right="0.071cm" fo:padding-top="0.035cm" style:vertical-align="middle"/>
       <style:text-properties fo:color="#000000" style:font-name="ArialMT" fo:font-size="11pt" style:font-name-asian="ArialMT" style:font-size-asian="11pt" style:font-name-complex="ArialMT" style:font-size-complex="11pt"/>
     </style:style>
@@ -315,7 +317,7 @@
         </table:table-row>
         <table:table-row table:style-name="ro2">
           <table:table-cell/>
-          <table:table-cell table:style-name="Sheet0_cell1" office:value-type="string" calcext:value-type="string">
+          <table:table-cell table:style-name="ce3" office:value-type="string" calcext:value-type="string">
             <text:p>
               <text:span text:style-name="T1">This document was exported from Numbers. Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</text:span>
             </text:p>
@@ -2037,54 +2039,218 @@
           </table:table-cell>
         </table:table-row>
         <table:table-row table:style-name="ro8">
-          <table:table-cell table:number-columns-repeated="8"/>
-          <table:table-cell table:formula="of:=IF(SUM([.B32:.F32];[.H32])=0;&quot;&quot;;SUM([.B32:.F32];[.H32]))">
-            <text:p/>
-          </table:table-cell>
-          <table:table-cell table:formula="of:=IF([.I32]=&quot;&quot;;&quot;&quot;;1440-[.I32])">
-            <text:p/>
-          </table:table-cell>
-          <table:table-cell table:number-columns-repeated="4"/>
-        </table:table-row>
-        <table:table-row table:style-name="ro8">
-          <table:table-cell table:number-columns-repeated="8"/>
-          <table:table-cell table:formula="of:=IF(SUM([.B33:.F33];[.H33])=0;&quot;&quot;;SUM([.B33:.F33];[.H33]))">
-            <text:p/>
-          </table:table-cell>
-          <table:table-cell table:formula="of:=IF([.I33]=&quot;&quot;;&quot;&quot;;1440-[.I33])">
-            <text:p/>
-          </table:table-cell>
-          <table:table-cell table:number-columns-repeated="4"/>
-        </table:table-row>
-        <table:table-row table:style-name="ro8">
-          <table:table-cell table:number-columns-repeated="8"/>
-          <table:table-cell table:formula="of:=IF(SUM([.B34:.F34];[.H34])=0;&quot;&quot;;SUM([.B34:.F34];[.H34]))">
-            <text:p/>
-          </table:table-cell>
-          <table:table-cell table:formula="of:=IF([.I34]=&quot;&quot;;&quot;&quot;;1440-[.I34])">
-            <text:p/>
-          </table:table-cell>
-          <table:table-cell table:number-columns-repeated="4"/>
-        </table:table-row>
-        <table:table-row table:style-name="ro8">
-          <table:table-cell table:number-columns-repeated="8"/>
-          <table:table-cell table:formula="of:=IF(SUM([.B35:.F35];[.H35])=0;&quot;&quot;;SUM([.B35:.F35];[.H35]))">
-            <text:p/>
-          </table:table-cell>
-          <table:table-cell table:formula="of:=IF([.I35]=&quot;&quot;;&quot;&quot;;1440-[.I35])">
-            <text:p/>
-          </table:table-cell>
-          <table:table-cell table:number-columns-repeated="4"/>
-        </table:table-row>
-        <table:table-row table:style-name="ro8">
-          <table:table-cell table:number-columns-repeated="8"/>
-          <table:table-cell table:formula="of:=IF(SUM([.B36:.F36];[.H36])=0;&quot;&quot;;SUM([.B36:.F36];[.H36]))">
-            <text:p/>
-          </table:table-cell>
-          <table:table-cell table:formula="of:=IF([.I36]=&quot;&quot;;&quot;&quot;;1440-[.I36])">
-            <text:p/>
-          </table:table-cell>
-          <table:table-cell table:number-columns-repeated="4"/>
+          <table:table-cell office:value-type="date" office:date-value="2026-09-12" calcext:value-type="date">
+            <text:p>12/09/2026</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="450" calcext:value-type="float">
+            <text:p>450</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="70" calcext:value-type="float">
+            <text:p>70</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="180" calcext:value-type="float">
+            <text:p>180</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="60" calcext:value-type="float">
+            <text:p>60</text:p>
+          </table:table-cell>
+          <table:table-cell table:number-columns-repeated="2" office:value-type="float" office:value="0" calcext:value-type="float">
+            <text:p>0</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="120" calcext:value-type="float">
+            <text:p>120</text:p>
+          </table:table-cell>
+          <table:table-cell table:style-name="ce37" table:formula="of:=IF(SUM([.B32:.F32];[.H32])=0;&quot;&quot;;SUM([.B32:.F32];[.H32]))" office:value-type="float" office:value="880" calcext:value-type="float">
+            <text:p>880</text:p>
+          </table:table-cell>
+          <table:table-cell table:style-name="ce37" table:formula="of:=IF([.I32]=&quot;&quot;;&quot;&quot;;1440-[.I32])" office:value-type="float" office:value="560" calcext:value-type="float">
+            <text:p>560</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Great</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Neutral</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>High</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Good</text:p>
+          </table:table-cell>
+        </table:table-row>
+        <table:table-row table:style-name="ro8">
+          <table:table-cell office:value-type="date" office:date-value="2026-09-13" calcext:value-type="date">
+            <text:p>13/09/2026</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="500" calcext:value-type="float">
+            <text:p>500</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="90" calcext:value-type="float">
+            <text:p>90</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="180" calcext:value-type="float">
+            <text:p>180</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="60" calcext:value-type="float">
+            <text:p>60</text:p>
+          </table:table-cell>
+          <table:table-cell table:number-columns-repeated="2" office:value-type="float" office:value="0" calcext:value-type="float">
+            <text:p>0</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="150" calcext:value-type="float">
+            <text:p>150</text:p>
+          </table:table-cell>
+          <table:table-cell table:style-name="ce37" table:formula="of:=IF(SUM([.B33:.F33];[.H33])=0;&quot;&quot;;SUM([.B33:.F33];[.H33]))" office:value-type="float" office:value="980" calcext:value-type="float">
+            <text:p>980</text:p>
+          </table:table-cell>
+          <table:table-cell table:style-name="ce37" table:formula="of:=IF([.I33]=&quot;&quot;;&quot;&quot;;1440-[.I33])" office:value-type="float" office:value="460" calcext:value-type="float">
+            <text:p>460</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Great</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Neutral</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>High</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Better</text:p>
+          </table:table-cell>
+        </table:table-row>
+        <table:table-row table:style-name="ro8">
+          <table:table-cell office:value-type="date" office:date-value="2026-09-14" calcext:value-type="date">
+            <text:p>14/09/2026</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="380" calcext:value-type="float">
+            <text:p>380</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="60" calcext:value-type="float">
+            <text:p>60</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="120" calcext:value-type="float">
+            <text:p>120</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="60" calcext:value-type="float">
+            <text:p>60</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="100" calcext:value-type="float">
+            <text:p>100</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="2" calcext:value-type="float">
+            <text:p>2</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="90" calcext:value-type="float">
+            <text:p>90</text:p>
+          </table:table-cell>
+          <table:table-cell table:style-name="ce37" table:formula="of:=IF(SUM([.B34:.F34];[.H34])=0;&quot;&quot;;SUM([.B34:.F34];[.H34]))" office:value-type="float" office:value="810" calcext:value-type="float">
+            <text:p>810</text:p>
+          </table:table-cell>
+          <table:table-cell table:style-name="ce37" table:formula="of:=IF([.I34]=&quot;&quot;;&quot;&quot;;1440-[.I34])" office:value-type="float" office:value="630" calcext:value-type="float">
+            <text:p>630</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Great</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Satisfied</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Medium</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Better</text:p>
+          </table:table-cell>
+        </table:table-row>
+        <table:table-row table:style-name="ro8">
+          <table:table-cell office:value-type="date" office:date-value="2026-09-15" calcext:value-type="date">
+            <text:p>15/09/2026</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="400" calcext:value-type="float">
+            <text:p>400</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="70" calcext:value-type="float">
+            <text:p>70</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="150" calcext:value-type="float">
+            <text:p>150</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="60" calcext:value-type="float">
+            <text:p>60</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="300" calcext:value-type="float">
+            <text:p>300</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="6" calcext:value-type="float">
+            <text:p>6</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="70" calcext:value-type="float">
+            <text:p>70</text:p>
+          </table:table-cell>
+          <table:table-cell table:style-name="ce37" table:formula="of:=IF(SUM([.B35:.F35];[.H35])=0;&quot;&quot;;SUM([.B35:.F35];[.H35]))" office:value-type="float" office:value="1050" calcext:value-type="float">
+            <text:p>1050</text:p>
+          </table:table-cell>
+          <table:table-cell table:style-name="ce37" table:formula="of:=IF([.I35]=&quot;&quot;;&quot;&quot;;1440-[.I35])" office:value-type="float" office:value="390" calcext:value-type="float">
+            <text:p>390</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Good</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Satisfied</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Medium</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Normal</text:p>
+          </table:table-cell>
+        </table:table-row>
+        <table:table-row table:style-name="ro8">
+          <table:table-cell office:value-type="date" office:date-value="2026-09-16" calcext:value-type="date">
+            <text:p>16/09/2026</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="350" calcext:value-type="float">
+            <text:p>350</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="70" calcext:value-type="float">
+            <text:p>70</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="180" calcext:value-type="float">
+            <text:p>180</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="60" calcext:value-type="float">
+            <text:p>60</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="400" calcext:value-type="float">
+            <text:p>400</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="8" calcext:value-type="float">
+            <text:p>8</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="float" office:value="80" calcext:value-type="float">
+            <text:p>80</text:p>
+          </table:table-cell>
+          <table:table-cell table:style-name="ce37" table:formula="of:=IF(SUM([.B36:.F36];[.H36])=0;&quot;&quot;;SUM([.B36:.F36];[.H36]))" office:value-type="float" office:value="1140" calcext:value-type="float">
+            <text:p>1140</text:p>
+          </table:table-cell>
+          <table:table-cell table:style-name="ce37" table:formula="of:=IF([.I36]=&quot;&quot;;&quot;&quot;;1440-[.I36])" office:value-type="float" office:value="300" calcext:value-type="float">
+            <text:p>300</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Stressed</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Unsatisfied</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Low</text:p>
+          </table:table-cell>
+          <table:table-cell office:value-type="string" calcext:value-type="string">
+            <text:p>Busy Day</text:p>
+          </table:table-cell>
         </table:table-row>
         <table:table-row table:style-name="ro8">
           <table:table-cell table:number-columns-repeated="8"/>
@@ -5747,10 +5913,10 @@
 <office:document-meta xmlns:grddl="http://www.w3.org/2003/g/data-view#" xmlns:meta="urn:oasis:names:tc:opendocument:xmlns:meta:1.0" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:xlink="http://www.w3.org/1999/xlink" xmlns:ooo="http://openoffice.org/2004/office" xmlns:office="urn:oasis:names:tc:opendocument:xmlns:office:1.0" office:version="1.4">
   <office:meta>
     <meta:generator>LibreOffice/26.8.0.3$MacOSX_AARCH64 LibreOffice_project/bce0998afefdbc355585ca324285661a2170ba77</meta:generator>
-    <dc:date>2026-09-11T23:46:01.657041000</dc:date>
-    <meta:editing-duration>PT9M26S</meta:editing-duration>
-    <meta:editing-cycles>1</meta:editing-cycles>
-    <meta:document-statistic meta:table-count="3" meta:cell-count="1164" meta:object-count="0"/>
+    <dc:date>2026-09-17T01:37:32.935889000</dc:date>
+    <meta:editing-duration>PT23M8S</meta:editing-duration>
+    <meta:editing-cycles>2</meta:editing-cycles>
+    <meta:document-statistic meta:table-count="3" meta:cell-count="1224" meta:object-count="0"/>
     <meta:user-defined meta:name=""/>
   </office:meta>
 </office:document-meta>
@@ -5769,15 +5935,15 @@
           <config:config-item config:name="ViewId" config:type="string">view1</config:config-item>
           <config:config-item-map-named config:name="Tables">
             <config:config-item-map-entry config:name="Daily Log_Table 1">
-              <config:config-item config:name="CursorPositionX" config:type="int">14</config:config-item>
-              <config:config-item config:name="CursorPositionY" config:type="int">30</config:config-item>
+              <config:config-item config:name="CursorPositionX" config:type="int">3</config:config-item>
+              <config:config-item config:name="CursorPositionY" config:type="int">34</config:config-item>
               <config:config-item config:name="ActiveSplitRange" config:type="short">2</config:config-item>
-              <config:config-item config:name="PositionLeft" config:type="int">7</config:config-item>
+              <config:config-item config:name="PositionLeft" config:type="int">0</config:config-item>
               <config:config-item config:name="PositionRight" config:type="int">0</config:config-item>
               <config:config-item config:name="PositionTop" config:type="int">0</config:config-item>
-              <config:config-item config:name="PositionBottom" config:type="int">6</config:config-item>
+              <config:config-item config:name="PositionBottom" config:type="int">26</config:config-item>
               <config:config-item config:name="ZoomType" config:type="short">0</config:config-item>
-              <config:config-item config:name="ZoomValue" config:type="int">100</config:config-item>
+              <config:config-item config:name="ZoomValue" config:type="int">110</config:config-item>
               <config:config-item config:name="PageViewZoomValue" config:type="int">60</config:config-item>
               <config:config-item config:name="ShowGrid" config:type="boolean">true</config:config-item>
               <config:config-item config:name="AnchoredTextOverflowLegacy" config:type="boolean">false</config:config-item>
@@ -5795,7 +5961,7 @@
               <config:config-item config:name="PositionTop" config:type="int">0</config:config-item>
               <config:config-item config:name="PositionBottom" config:type="int">0</config:config-item>
               <config:config-item config:name="ZoomType" config:type="short">0</config:config-item>
-              <config:config-item config:name="ZoomValue" config:type="int">100</config:config-item>
+              <config:config-item config:name="ZoomValue" config:type="int">110</config:config-item>
               <config:config-item config:name="PageViewZoomValue" config:type="int">60</config:config-item>
               <config:config-item config:name="ShowGrid" config:type="boolean">true</config:config-item>
               <config:config-item config:name="AnchoredTextOverflowLegacy" config:type="boolean">false</config:config-item>
@@ -5806,9 +5972,9 @@
             </config:config-item-map-entry>
           </config:config-item-map-named>
           <config:config-item config:name="ActiveTable" config:type="string">Daily Log_Table 1</config:config-item>
-          <config:config-item config:name="HorizontalScrollbarWidth" config:type="int">1377</config:config-item>
+          <config:config-item config:name="HorizontalScrollbarWidth" config:type="int">1357</config:config-item>
           <config:config-item config:name="ZoomType" config:type="short">0</config:config-item>
-          <config:config-item config:name="ZoomValue" config:type="int">100</config:config-item>
+          <config:config-item config:name="ZoomValue" config:type="int">110</config:config-item>
           <config:config-item config:name="PageViewZoomValue" config:type="int">60</config:config-item>
           <config:config-item config:name="ShowPageBreakPreview" config:type="boolean">false</config:config-item>
           <config:config-item config:name="ShowZeroValues" config:type="boolean">true</config:config-item>
@@ -5830,7 +5996,7 @@
           <config:config-item config:name="RasterSubdivisionY" config:type="int">1</config:config-item>
           <config:config-item config:name="IsRasterAxisSynchronized" config:type="boolean">true</config:config-item>
           <config:config-item config:name="FormulaBarHeight" config:type="short">1</config:config-item>
-          <config:config-item config:name="WindowState" config:type="string">-1,62,1440,780;1;0,0,1440,900;</config:config-item>
+          <config:config-item config:name="WindowState" config:type="string">0,62,1420,751;1;,,,;</config:config-item>
           <config:config-item config:name="AnchoredTextOverflowLegacy" config:type="boolean">false</config:config-item>
           <config:config-item config:name="LegacySingleLineFontwork" config:type="boolean">false</config:config-item>
           <config:config-item config:name="ConnectorUseSnapRect" config:type="boolean">false</config:config-item>
@@ -5861,9 +6027,9 @@
       <config:config-item config:name="LinkUpdateMode" config:type="short">3</config:config-item>
       <config:config-item config:name="LoadReadonly" config:type="boolean">false</config:config-item>
       <config:config-item config:name="ModifyPasswordHash" config:type="int">0</config:config-item>
-      <config:config-item config:name="PrinterName" config:type="string"/>
+      <config:config-item config:name="PrinterName" config:type="string">Default printer</config:config-item>
       <config:config-item config:name="PrinterPaperFromSetup" config:type="boolean">false</config:config-item>
-      <config:config-item config:name="PrinterSetup" config:type="base64Binary"/>
+      <config:config-item config:name="PrinterSetup" config:type="base64Binary">FQH+/0RlZmF1bHQgcHJpbnRlcgAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAWAAQABAAAAAAAAAAEAAhSAAAEdAAAAAAAABIAQ09NUEFUX0RVUExFWF9NT0RFEwBEdXBsZXhNb2RlOjpVbmtub3duDABQUklOVEVSX05BTUUPAERlZmF1bHQgcHJpbnRlcgsARFJJVkVSX05BTUUAAA==</config:config-item>
       <config:config-item config:name="RasterIsVisible" config:type="boolean">false</config:config-item>
       <config:config-item config:name="RasterResolutionX" config:type="int">1000</config:config-item>
       <config:config-item config:name="RasterResolutionY" config:type="int">1000</config:config-item>
@@ -5905,8 +6071,6 @@
     <style:font-face style:name="ArialMT" svg:font-family="ArialMT"/>
     <style:font-face style:name="Calibri" svg:font-family="Calibri"/>
     <style:font-face style:name="Liberation Sans" svg:font-family="'Liberation Sans'" style:font-family-generic="swiss" style:font-pitch="variable"/>
-    <style:font-face style:name="Liberation Serif" svg:font-family="'Liberation Serif'" style:font-family-generic="roman" style:font-pitch="variable"/>
-    <style:font-face style:name="Tahoma" svg:font-family="Tahoma" style:font-family-generic="system" style:font-pitch="variable"/>
   </office:font-face-decls>
   <office:styles>
     <style:default-style style:family="table-cell">
@@ -5916,10 +6080,10 @@
     </style:default-style>
     <style:default-style style:family="graphic">
       <style:graphic-properties draw:stroke="none" svg:stroke-color="#3465a4" draw:fill-color="#ffffff" fo:wrap-option="wrap" draw:shadow="hidden" draw:shadow-offset-x="0.3cm" draw:shadow-offset-y="0.3cm" style:writing-mode="page"/>
-      <style:paragraph-properties style:text-autospace="ideograph-alpha" style:punctuation-wrap="simple" style:line-break="strict" style:font-independent-line-spacing="false">
+      <style:paragraph-properties style:text-autospace="ideograph-alpha" style:punctuation-wrap="simple" style:line-break="strict" loext:tab-stop-distance="0cm" style:font-independent-line-spacing="false">
         <style:tab-stops/>
       </style:paragraph-properties>
-      <style:text-properties style:use-window-font-color="true" loext:opacity="0%" style:font-name="Liberation Serif" fo:font-size="12pt" fo:language="en" fo:country="IN" style:letter-kerning="true" style:font-name-asian="Tahoma" style:font-size-asian="12pt" style:language-asian="zh" style:country-asian="CN" style:font-name-complex="Tahoma" style:font-size-complex="12pt" style:language-complex="hi" style:country-complex="IN"/>
+      <style:text-properties style:use-window-font-color="true" loext:opacity="0%" fo:font-family="'Liberation Serif'" style:font-family-generic="roman" style:font-pitch="variable" fo:font-size="12pt" fo:language="en" fo:country="IN" style:letter-kerning="true" style:font-family-asian="Tahoma" style:font-family-generic-asian="system" style:font-pitch-asian="variable" style:font-size-asian="12pt" style:language-asian="zh" style:country-asian="CN" style:font-family-complex="Tahoma" style:font-family-generic-complex="system" style:font-pitch-complex="variable" style:font-size-complex="12pt" style:language-complex="hi" style:country-complex="IN"/>
     </style:default-style>
     <style:style style:name="Default" style:family="graphic"/>
     <style:style style:name="Note" style:family="graphic" style:parent-style-name="Default">
@@ -6080,9 +6244,9 @@
         </style:region-left>
         <style:region-right>
           <text:p>
-            <text:date style:data-style-name="N2" text:date-value="2026-09-11">00/00/0000</text:date>
+            <text:date style:data-style-name="N2" text:date-value="2026-09-17">00/00/0000</text:date>
             , 
-            <text:time>00:00:00</text:time>
+            <text:time style:data-style-name="N2" text:time-value="01:23:50.824636000">00:00:00</text:time>
           </text:p>
         </style:region-right>
       </style:header>

</xml_diff>